<commit_message>
Corrige o mecanismo causal da aba Dispersão de preço
O passo 4 da cadeia anterior assumia que o consumidor clicava no aviso de
"outros vendedores" e migrava para a oferta mais barata. A premissa está
errada: a Buy Box concentra a esmagadora maioria das vendas de um ASIN e o
link de outras ofertas é caminho de baixíssimo tráfego.

O mecanismo correto é a própria Amazon reagindo a uma oferta FBA 39% mais
barata no mesmo ASIN — perdendo a Buy Box para o terceiro ou deixando de
comprar um item em que seu custo não compete. A perda de Buy Box neste
catálogo está provada por print: na Bica Pedra, com selo Escolha da Amazon,
quem detém a Buy Box é a Cobasi.

Cada passo agora carrega o nível de evidência (print, declarado na call ou
inferência). Adicionada nota explicando por que a Buy Box reposiciona dois
achados da planilha como perda quase total.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017xRPoJqxsuGFv4VmDesebx
</commit_message>
<xml_diff>
--- a/stillpet/Evidencias_StillPet_Amazon_BR_2026-09-23.xlsx
+++ b/stillpet/Evidencias_StillPet_Amazon_BR_2026-09-23.xlsx
@@ -4068,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G30"/>
+  <dimension ref="A2:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4241,84 +4241,118 @@
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>HIPOTESE DE CAUSA - NAO CONFIRMADA, NAO LEVAR AO DECK SEM O CARLOS CONFIRMAR</t>
+          <t>MECANISMO - cada passo marcado com o nivel de evidencia. NAO levar ao deck sem o Carlos confirmar os passos 1 e 2.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>1. Na call, a Beatriz declarou que a Amazon exigia desconto de 8% a 11% e que a StillPet 'subia um pouco o preco justamente para ter esse desconto'.</t>
+          <t>1. Na call, a Beatriz declarou que a Amazon exigia desconto de 8% a 11% e que a StillPet 'subia um pouco o preco justamente para ter esse desconto'.  [DECLARADO NA CALL]</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2. A Amazon monta a margem dela sobre um custo ja inflado - o 1P chega a R$18,32.</t>
+          <t>2. A Amazon monta a margem dela sobre um custo ja inflado - o 1P chega a R$18,32.  [INFERENCIA]</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>3. Um revendedor compra no atacado normal e lista via FBA a R$11,25, com margem.</t>
+          <t>3. Um revendedor compra no atacado normal e lista via FBA a R$11,25, com margem.  [PRINT 23/09/2026]</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>4. A propria pagina da Amazon avisa o comprador que existe mais barato ao lado.</t>
+          <t>4. O mecanismo NAO e o consumidor clicar em 'outros vendedores' - a Buy Box concentra a esmagadora maioria das vendas na Amazon, e o link de outras ofertas e caminho de baixissimo trafego.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>5. O ASIN 1P perde venda, e o algoritmo de compra da Amazon reduz o pedido de reposicao.</t>
+          <t>5. O mecanismo e a propria Amazon: diante de uma oferta FBA 39% mais barata no mesmo ASIN, ou ela perde a Buy Box para o terceiro, ou deixa de comprar um item em que seu custo nao compete.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>6. Foi exatamente o que a StillPet descreveu: o produto que representava 60-70% da venda na Amazon caiu.</t>
+          <t>6. PERDER A BUY BOX NESTE CATALOGO ESTA PROVADO: na Bica Pedra Calopsitas, com selo Escolha da Amazon, quem detem a Buy Box e a Cobasi - nao a Amazon.  [PRINT 23/09/2026]</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>7. A conclusao da fabrica virou 'a Amazon e burocratica e nao funciona'. A evidencia aponta para arquitetura de preco, nao burocracia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="5" t="inlineStr">
+          <t>7. A reducao de pedido de reposicao por falta de competitividade de preco e INFERENCIA - coerente com o relato da fabrica, mas nao verificada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>8. Foi o que a StillPet descreveu: o produto que representava 60-70% da venda na Amazon caiu.  [DECLARADO NA CALL]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>9. A conclusao da fabrica virou 'a Amazon e burocratica e nao funciona'. A evidencia aponta para arquitetura de preco, nao burocracia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>RESTRICAO LEGAL - Lei 12.529/2011</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="6" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Monitorar preco e orientar posicionamento: pode. Impor preco minimo de revenda com punicao: NAO. A correcao aqui e no preco de sell-in que a StillPet pratica com a Amazon e com os distribuidores - o que e 100% legal e 100% sob controle dela. Nunca escrever 'MAP enforcement', 'preco minimo aplicado' ou 'garantimos que ninguem venda abaixo de X'.</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>POR QUE A BUY BOX E O ATIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>A Buy Box concentra a esmagadora maioria das vendas de um ASIN. Isso reposiciona dois achados desta planilha como perda quase total, nao parcial: (a) o Comedouro Filhote 450ml Rosa, com 4,8 estrelas e 182 avaliacoes, esta SEM Buy Box - nao e venda reduzida, e venda proxima de zero; (b) na Bica Pedra, com selo Escolha da Amazon, quem detem a Buy Box e a Cobasi - ou seja, praticamente toda a venda desse ASIN e da Cobasi. Se for usar um percentual de Buy Box no deck, cite a fonte do estudo - nao publique numero sem referencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="B14:G16"/>
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B22:G22"/>
-    <mergeCell ref="B28:G30"/>
     <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B30:G32"/>
+    <mergeCell ref="B36:G39"/>
+    <mergeCell ref="B26:G26"/>
     <mergeCell ref="B21:G21"/>
     <mergeCell ref="B25:G25"/>
   </mergeCells>

</xml_diff>